<commit_message>
Update final report materials
</commit_message>
<xml_diff>
--- a/reports/stage9_report_materials/stage9_tables.xlsx
+++ b/reports/stage9_report_materials/stage9_tables.xlsx
@@ -187,7 +187,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="10477500" cy="5905500"/>
+    <ext cx="10477500" cy="5876925"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -708,10 +708,10 @@
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -766,22 +766,22 @@
         <v>1</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>0.54</v>
+        <v>0.84</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>0.857</v>
+        <v>0.9595</v>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.2525</v>
+        <v>0.5</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>0.26</v>
+        <v>0.915</v>
       </c>
       <c r="G2" s="2" t="n">
-        <v>0.08500000000000001</v>
+        <v>0.225</v>
       </c>
       <c r="H2" s="2" t="n">
-        <v>0</v>
+        <v>0.55</v>
       </c>
     </row>
     <row r="3">
@@ -794,22 +794,22 @@
         <v>1</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>0.51</v>
+        <v>0.955</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>0.847</v>
+        <v>0.995</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.2275</v>
+        <v>0.5308333333333334</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>0.23</v>
+        <v>0.915</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>0.06</v>
+        <v>0.285</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>0</v>
+        <v>0.59</v>
       </c>
     </row>
     <row r="4">
@@ -837,7 +837,7 @@
         <v>0.11</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0</v>
+        <v>0.11</v>
       </c>
     </row>
     <row r="5">
@@ -865,7 +865,7 @@
         <v>0.36</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0</v>
+        <v>0.4186046511627907</v>
       </c>
     </row>
     <row r="6">
@@ -912,7 +912,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="21" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
@@ -952,10 +952,10 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>0.18079</v>
+        <v>0.331945</v>
       </c>
       <c r="C2" s="2" t="n">
-        <v>106.309</v>
+        <v>108.227</v>
       </c>
       <c r="D2" s="2" t="n">
         <v>0</v>
@@ -971,10 +971,10 @@
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.32999</v>
+        <v>0.396755</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>210.348</v>
+        <v>220.566</v>
       </c>
       <c r="D3" s="2" t="n">
         <v>0</v>
@@ -989,15 +989,11 @@
           <t>B2</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
-        <is>
-          <t>нет замера</t>
-        </is>
-      </c>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>нет замера</t>
-        </is>
+      <c r="B4" s="2" t="n">
+        <v>3.58689</v>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>108.402</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
Refresh benchmark notebooks and report materials
</commit_message>
<xml_diff>
--- a/reports/stage9_report_materials/stage9_tables.xlsx
+++ b/reports/stage9_report_materials/stage9_tables.xlsx
@@ -707,11 +707,11 @@
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
     <col width="20" customWidth="1" min="5" max="5"/>
     <col width="13" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -822,22 +822,22 @@
         <v>1</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>0.62</v>
+        <v>0.855</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>0.8703333333333333</v>
+        <v>0.973</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.11</v>
+        <v>0.5766666666666667</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>0.11</v>
+        <v>0.92</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>0.11</v>
+        <v>0.22</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>0.11</v>
+        <v>0.22</v>
       </c>
     </row>
     <row r="5">
@@ -847,25 +847,25 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>0.5</v>
+        <v>0.84</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.7533333333333333</v>
+        <v>0.92</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.59</v>
+        <v>0.5533333333333333</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>0.84</v>
+        <v>0.66</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>0.36</v>
+        <v>0.28</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>0.4186046511627907</v>
+        <v>0.28</v>
       </c>
     </row>
     <row r="6">
@@ -878,22 +878,22 @@
         <v>0.95</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>0.5</v>
+        <v>0.9</v>
       </c>
       <c r="D6" s="2" t="n">
-        <v>0.8</v>
+        <v>0.95</v>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.5</v>
+        <v>0.5333333333333333</v>
       </c>
       <c r="F6" s="2" t="n">
-        <v>0.85</v>
+        <v>0.75</v>
       </c>
       <c r="G6" s="2" t="n">
-        <v>0.5</v>
+        <v>0.3</v>
       </c>
       <c r="H6" s="2" t="n">
-        <v>0.5</v>
+        <v>0.35</v>
       </c>
     </row>
   </sheetData>
@@ -990,10 +990,10 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>3.58689</v>
+        <v>7.05238</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>108.402</v>
+        <v>109.949</v>
       </c>
       <c r="D4" s="2" t="n">
         <v>0</v>
@@ -1009,13 +1009,13 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>10187.22126</v>
+        <v>20101.22146</v>
       </c>
       <c r="C5" s="2" t="n">
-        <v>1983.812</v>
+        <v>1981.508</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>0.14</v>
+        <v>0.08</v>
       </c>
       <c r="E5" s="2" t="n">
         <v>50</v>
@@ -1028,10 +1028,10 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>34898.12519999999</v>
+        <v>66825.6801</v>
       </c>
       <c r="C6" s="2" t="n">
-        <v>2153.457</v>
+        <v>2127.145</v>
       </c>
       <c r="D6" s="2" t="n">
         <v>0.05</v>

</xml_diff>

<commit_message>
Fix Colab waiter and refresh Stage 9 materials
</commit_message>
<xml_diff>
--- a/reports/stage9_report_materials/stage9_tables.xlsx
+++ b/reports/stage9_report_materials/stage9_tables.xlsx
@@ -157,7 +157,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="9906000" cy="5133975"/>
+    <ext cx="9906000" cy="5095875"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -497,15 +497,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F6"/>
+  <dimension ref="A1:F10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="37" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="31" customWidth="1" min="5" max="5"/>
-    <col width="39" customWidth="1" min="6" max="6"/>
+    <col width="42" customWidth="1" min="5" max="5"/>
+    <col width="42" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -687,6 +687,126 @@
       <c r="F6" s="2" t="inlineStr">
         <is>
           <t>3 кандидата + validator/reranker</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>B5a</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>B5_stage8_qwen3_14b</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Stage 8 LLM + strict JSON validator</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>stage8_qwen3_14b_sample20</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Qwen3-14B, один кандидат, validator retry</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>B5b</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>B5_stage8_mistral_small_32_24b_bnb4</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Stage 8 LLM + strict JSON validator</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>stage8_mistral_small_32_24b_bnb4_sample20</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Mistral Small 3.2 24B bnb-4bit, один кандидат</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>B5c</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>B5_stage8_gemma3_12b_it</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Stage 8 LLM + strict JSON validator</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>stage8_gemma3_12b_it_sample20</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Gemma 3 12B IT, gated HF model</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>B5d</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>B5_stage8_gemma4_e2b_it</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Stage 8 LLM + strict JSON validator</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>stage8_gemma4_e2b_it_sample20</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Gemma 4 E2B IT, малый контрольный LLM baseline</t>
         </is>
       </c>
     </row>
@@ -701,7 +821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H6"/>
+  <dimension ref="A1:H10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -896,6 +1016,118 @@
         <v>0.35</v>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>B5a</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>0.575</v>
+      </c>
+      <c r="F7" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="G7" s="2" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>B5b</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F8" s="2" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="G8" s="2" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>B5c</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>0.075</v>
+      </c>
+      <c r="F9" s="2" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="G9" s="2" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>B5d</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>0.89</v>
+      </c>
+      <c r="E10" s="2" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F10" s="2" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="G10" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -908,7 +1140,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1037,6 +1269,82 @@
         <v>0.05</v>
       </c>
       <c r="E6" s="2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>B5a</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>8133.003999999999</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>2064.027</v>
+      </c>
+      <c r="D7" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>B5b</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>6045.25885</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>1889.961</v>
+      </c>
+      <c r="D8" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>B5c</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>69237.62940000001</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2556.523</v>
+      </c>
+      <c r="D9" s="2" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>B5d</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>44562.2476</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>2200</v>
+      </c>
+      <c r="D10" s="2" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="E10" s="2" t="n">
         <v>20</v>
       </c>
     </row>
@@ -1052,7 +1360,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -1190,6 +1498,94 @@
       <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Три генерации на пример; примерно в 3.4 раза медленнее B3</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>B5a</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Лучший протестированный одиночный LLM baseline на Stage 8</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Qwen3-14B дает 100% validity и сильные метрики без reranking</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Проверен на sample20; медленнее детерминированных B0-B2</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>B5b</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Быстрый Stage 8 LLM baseline с квантизованным Mistral Small 3.2</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Хороший компромисс скорости и валидности</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Уступает Qwen3-14B по chart type и exact match</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>B5c</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Отрицательный контроль для Gemma 3 12B в текущем prompt/schema режиме</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Показывает риск gated VLM/LLM без точной настройки JSON-формата</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>85% failed на sample20; не рекомендуется как baseline без доработки промпта</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>B5d</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Малый контрольный Stage 8 LLM baseline</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Показывает нижнюю границу качества для малой Gemma</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Хуже Qwen3-14B и Mistral Small 3.2 по основным метрикам</t>
         </is>
       </c>
     </row>
@@ -1204,10 +1600,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C6"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="37" customWidth="1" min="1" max="1"/>
     <col width="42" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
   </cols>
@@ -1254,7 +1650,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>B3/B4 медленнее детерминированных базовых подходов</t>
+          <t>B3/B4/B5 медленнее детерминированных базовых подходов</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
@@ -1266,49 +1662,83 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Ошибки рендеринга</t>
+          <t>Разные размеры выборок</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Некоторые валидные specs могут не отрендериться</t>
+          <t>B0-B2 посчитаны на sample200, B3 на sample50, B4/B5 на sample20</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Сохранять render_failures.json и визуально проверять примеры</t>
+          <t>Явно показывать Sample в таблицах и не делать вывод о победе без полного прогона</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Несовместимость NL4DV</t>
+          <t>Нестабильность JSON у отдельных LLM</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Полный базовый подход на существующем инструменте не был установлен</t>
+          <t>Gemma 3 12B показала высокий failure rate в текущем Stage 8 контуре</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Зафиксировать dependency conflict и использовать B2 как частичный резервный вариант</t>
+          <t>Использовать строгий validator/retry и отдельно дорабатывать chat template/prompt</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>Ошибки рендеринга</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Некоторые валидные specs могут не отрендериться</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Сохранять render_failures.json и визуально проверять примеры</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Несовместимость NL4DV</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Полный базовый подход на существующем инструменте не был установлен</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Зафиксировать dependency conflict и использовать B2 как частичный резервный вариант</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
           <t>Нет оценки Text-to-SQL</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="B8" s="2" t="inlineStr">
         <is>
           <t>Качество upstream SQL здесь не измеряется</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Явно фиксировать границу post-query постановки</t>
         </is>

</xml_diff>